<commit_message>
Reemplaza el backlog CSV por el archivo .reqw de ReqView
</commit_message>
<xml_diff>
--- a/U4A1-Trazabilidad/Matriz_trazabilidad.xlsx
+++ b/U4A1-Trazabilidad/Matriz_trazabilidad.xlsx
@@ -526,7 +526,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fuentes: backlog (Backlog/Product_backlog_ReqView.csv), código (marcas @trace en U3A2-Prototipado/prototipo/index.html), pruebas (U3A2-Prototipado/pruebas/resultados_pruebas.json),</t>
+          <t>Fuentes: backlog (Backlog/Product_backlog.reqw), código (marcas @trace en U3A2-Prototipado/prototipo/index.html), pruebas (U3A2-Prototipado/pruebas/resultados_pruebas.json),</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4522,7 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Backlog/Product_backlog.html
-Backlog/Product_backlog_ReqView.csv</t>
+Backlog/Product_backlog.reqw</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">

</xml_diff>